<commit_message>
Add painting work section to BOQ
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192fkqnFqH7S7Jt3MJ4AXan
</commit_message>
<xml_diff>
--- a/boq/BOQ_OhmHouse.xlsx
+++ b/boq/BOQ_OhmHouse.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1570,36 +1570,98 @@
       </c>
       <c r="G48" s="8" t="n"/>
     </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>9. งานสี</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
+      <c r="F49" s="5" t="n"/>
+      <c r="G49" s="5" t="n"/>
+    </row>
     <row r="50">
-      <c r="A50" s="10" t="n"/>
-      <c r="B50" s="10" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>สีทาบ้าน (ผนัง 2 หน้า 381.10 ตร.ม. + ฝ้า 129.82 ตร.ม. = 510.92 ตร.ม., ถังละ 60 ตร.ม.)</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>ถัง (17.5ลิตร)</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>700</v>
+      </c>
+      <c r="F50" s="7">
+        <f>C50*E50</f>
+        <v/>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>สีเกรดประหยัด ทา 2 รอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>รวม หมวด 9 งานสี</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="n"/>
+      <c r="D51" s="8" t="n"/>
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="9" t="n">
+        <v>6300</v>
+      </c>
+      <c r="G51" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="n"/>
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>รวมทั้งหมดทุกหมวด (Grand Total)</t>
         </is>
       </c>
-      <c r="C50" s="10" t="n"/>
-      <c r="D50" s="10" t="n"/>
-      <c r="E50" s="10" t="n"/>
-      <c r="F50" s="11" t="n">
-        <v>547654</v>
-      </c>
-      <c r="G50" s="10" t="n"/>
+      <c r="C53" s="10" t="n"/>
+      <c r="D53" s="10" t="n"/>
+      <c r="E53" s="10" t="n"/>
+      <c r="F53" s="11" t="n">
+        <v>553954</v>
+      </c>
+      <c r="G53" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="21">
     <mergeCell ref="A42:G42"/>
+    <mergeCell ref="B51:E51"/>
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B50:E50"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A49:G49"/>
     <mergeCell ref="B22:E22"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="A46:G46"/>
+    <mergeCell ref="B53:E53"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
Add stairs and MEP prep (plumbing, electrical main, waterproofing, gutter, grille/screen) to BOQ
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192fkqnFqH7S7Jt3MJ4AXan
</commit_message>
<xml_diff>
--- a/boq/BOQ_OhmHouse.xlsx
+++ b/boq/BOQ_OhmHouse.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1630,23 +1630,373 @@
       </c>
       <c r="G51" s="8" t="n"/>
     </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>10. บันได</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="5" t="n"/>
+      <c r="D52" s="5" t="n"/>
+      <c r="E52" s="5" t="n"/>
+      <c r="F52" s="5" t="n"/>
+      <c r="G52" s="5" t="n"/>
+    </row>
     <row r="53">
-      <c r="A53" s="10" t="n"/>
-      <c r="B53" s="10" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>คอนกรีตบันได (หน้า 4x1.05ม. + หลัง 1x0.84ม., หนา 0.25ม.)</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>ลบ.ม.</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F53" s="7">
+        <f>C53*E53</f>
+        <v/>
+      </c>
+      <c r="G53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>เหล็กเสริมบันได DB9 (ประมาณ)</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>กก.</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F54" s="7">
+        <f>C54*E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="5" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>กระเบื้องปูขั้นบันได+ลูกตั้ง (+10% เผื่อเสีย)</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>ตร.ม.</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="F55" s="7">
+        <f>C55*E55</f>
+        <v/>
+      </c>
+      <c r="G55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n"/>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>รวม หมวด 10 บันได</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="8" t="n"/>
+      <c r="E56" s="8" t="n"/>
+      <c r="F56" s="9" t="n">
+        <v>7186</v>
+      </c>
+      <c r="G56" s="8" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>11. งานระบบ (ประปา/ไฟเมน/กันซึม/รางน้ำ/เหล็กดัด)</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n"/>
+      <c r="C57" s="5" t="n"/>
+      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="5" t="n"/>
+      <c r="F57" s="5" t="n"/>
+      <c r="G57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>งานประปา (เหมาจุด ท่อน้ำดี-เสีย สุขาภิบาล)</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>จุด</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>700</v>
+      </c>
+      <c r="F58" s="7">
+        <f>C58*E58</f>
+        <v/>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>~2 ห้องน้ำ + จุดนอกบ้าน</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>บ่อเกรอะ (ท่อวงซีเมนต์ 3 วง/ชุด x2 ชุด)</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>วง</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="F59" s="7">
+        <f>C59*E59</f>
+        <v/>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>ถูกกว่าถังบำบัดสำเร็จรูป</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>ถังเก็บน้ำ+ปั๊มน้ำอัตโนมัติ (เกรดประหยัด)</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>ชุด</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F60" s="7">
+        <f>C60*E60</f>
+        <v/>
+      </c>
+      <c r="G60" s="5" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>ตู้คอนซูมเมอร์ยูนิต+สายเมนไฟฟ้าเข้าบ้าน</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>ชุด</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F61" s="7">
+        <f>C61*E61</f>
+        <v/>
+      </c>
+      <c r="G61" s="5" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>น้ำยากันซึมห้องน้ำ (พื้น+ผนังสูง 1ม.)</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>31.52</v>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>ตร.ม.</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="F62" s="7">
+        <f>C62*E62</f>
+        <v/>
+      </c>
+      <c r="G62" s="5" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>11.6</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>รางน้ำฝนสังกะสี 4 นิ้ว + ติดตั้ง (รอบชายคา)</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>51.34</v>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>เมตร</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="F63" s="7">
+        <f>C63*E63</f>
+        <v/>
+      </c>
+      <c r="G63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>เหล็กดัด+มุ้งลวดหน้าต่างทุกบาน (18 บาน)</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>21.09</v>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>ตร.ม.</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>800</v>
+      </c>
+      <c r="F64" s="7">
+        <f>C64*E64</f>
+        <v/>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>เหล็กดัด 500 + มุ้งลวด 300 บาท/ตร.ม.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n"/>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>รวม หมวด 11 งานระบบ</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="n"/>
+      <c r="D65" s="8" t="n"/>
+      <c r="E65" s="8" t="n"/>
+      <c r="F65" s="9" t="n">
+        <v>63630</v>
+      </c>
+      <c r="G65" s="8" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="n"/>
+      <c r="B67" s="10" t="inlineStr">
         <is>
           <t>รวมทั้งหมดทุกหมวด (Grand Total)</t>
         </is>
       </c>
-      <c r="C53" s="10" t="n"/>
-      <c r="D53" s="10" t="n"/>
-      <c r="E53" s="10" t="n"/>
-      <c r="F53" s="11" t="n">
-        <v>553954</v>
-      </c>
-      <c r="G53" s="10" t="n"/>
+      <c r="C67" s="10" t="n"/>
+      <c r="D67" s="10" t="n"/>
+      <c r="E67" s="10" t="n"/>
+      <c r="F67" s="11" t="n">
+        <v>624770</v>
+      </c>
+      <c r="G67" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="25">
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="A52:G52"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B51:E51"/>
     <mergeCell ref="B32:E32"/>
@@ -1657,14 +2007,16 @@
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A49:G49"/>
     <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B56:E56"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="A46:G46"/>
-    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B67:E67"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A57:G57"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A23:G23"/>

</xml_diff>

<commit_message>
Switch septic to prefab tank (ถังแซท) instead of concrete rings
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192fkqnFqH7S7Jt3MJ4AXan
</commit_message>
<xml_diff>
--- a/boq/BOQ_OhmHouse.xlsx
+++ b/boq/BOQ_OhmHouse.xlsx
@@ -1795,19 +1795,19 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>บ่อเกรอะ (ท่อวงซีเมนต์ 3 วง/ชุด x2 ชุด)</t>
+          <t>ถังแซท (ถังบำบัดน้ำเสียสำเร็จรูป 600 ลิตร)</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>วง</t>
+          <t>ถัง</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
-        <v>240</v>
+        <v>2590</v>
       </c>
       <c r="F59" s="7">
         <f>C59*E59</f>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>ถูกกว่าถังบำบัดสำเร็จรูป</t>
+          <t>1 ถัง/ห้องน้ำ</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
       <c r="D65" s="8" t="n"/>
       <c r="E65" s="8" t="n"/>
       <c r="F65" s="9" t="n">
-        <v>63630</v>
+        <v>67370</v>
       </c>
       <c r="G65" s="8" t="n"/>
     </row>
@@ -1989,7 +1989,7 @@
       <c r="D67" s="10" t="n"/>
       <c r="E67" s="10" t="n"/>
       <c r="F67" s="11" t="n">
-        <v>624770</v>
+        <v>628510</v>
       </c>
       <c r="G67" s="10" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add contractor labor cost (2,400 baht/sqm, owner supplies materials)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192fkqnFqH7S7Jt3MJ4AXan
</commit_message>
<xml_diff>
--- a/boq/BOQ_OhmHouse.xlsx
+++ b/boq/BOQ_OhmHouse.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1978,24 +1978,85 @@
       </c>
       <c r="G65" s="8" t="n"/>
     </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>12. ค่าแรงเหมาช่าง (เจ้าของบ้านซื้อวัสดุเอง)</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
+      <c r="G66" s="5" t="n"/>
+    </row>
     <row r="67">
-      <c r="A67" s="10" t="n"/>
-      <c r="B67" s="10" t="inlineStr">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>ค่าแรงเหมาช่าง (ผู้รับเหมาคิดเฉพาะแรงงาน)</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="n">
+        <v>130</v>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>ตร.ม.</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F67" s="7">
+        <f>C67*E67</f>
+        <v/>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>เจ้าของบ้านซื้อวัสดุเองตามหมวด 1-11 ทั้งหมด</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n"/>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>รวม หมวด 12 ค่าแรงเหมาช่าง</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="n"/>
+      <c r="D68" s="8" t="n"/>
+      <c r="E68" s="8" t="n"/>
+      <c r="F68" s="9" t="n">
+        <v>312000</v>
+      </c>
+      <c r="G68" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="n"/>
+      <c r="B70" s="10" t="inlineStr">
         <is>
           <t>รวมทั้งหมดทุกหมวด (Grand Total)</t>
         </is>
       </c>
-      <c r="C67" s="10" t="n"/>
-      <c r="D67" s="10" t="n"/>
-      <c r="E67" s="10" t="n"/>
-      <c r="F67" s="11" t="n">
-        <v>628510</v>
-      </c>
-      <c r="G67" s="10" t="n"/>
+      <c r="C70" s="10" t="n"/>
+      <c r="D70" s="10" t="n"/>
+      <c r="E70" s="10" t="n"/>
+      <c r="F70" s="11" t="n">
+        <v>940510</v>
+      </c>
+      <c r="G70" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="27">
     <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B68:E68"/>
     <mergeCell ref="A52:G52"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="B51:E51"/>
@@ -2009,10 +2070,11 @@
     <mergeCell ref="B22:E22"/>
     <mergeCell ref="B56:E56"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B70:E70"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="A46:G46"/>
-    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="A66:G66"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="A2:G2"/>

</xml_diff>